<commit_message>
feat(govt): add LTN zero-coupon spread calculation and integrate compute_spreads_ltn
</commit_message>
<xml_diff>
--- a/datos_y_modelos/Domestic/domestic_sovereign_curve_brazil.xlsx
+++ b/datos_y_modelos/Domestic/domestic_sovereign_curve_brazil.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsiqueira4\Downloads\spread-model-master\light_spread-model-master\datos_y_modelos\Domestic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA68573-8AD5-4924-8A30-0A583257DA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CEF396-2321-48ED-88FF-28E086A778BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="18470" windowHeight="12220" xr2:uid="{4FA8D609-CF7D-453F-9379-B1555420C1B0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{4FA8D609-CF7D-453F-9379-B1555420C1B0}"/>
   </bookViews>
   <sheets>
     <sheet name="db_values_only" sheetId="1" r:id="rId1"/>
@@ -1050,7 +1050,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1060,6 +1060,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1077,13 +1083,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3324,7 +3331,7 @@
       <c r="M2">
         <v>712</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O2" t="s">
@@ -3437,7 +3444,7 @@
       <c r="M3">
         <v>1171</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O3" t="s">
@@ -3550,7 +3557,7 @@
       <c r="M4">
         <v>712</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O4" t="s">
@@ -3663,7 +3670,7 @@
       <c r="M5">
         <v>712</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O5" t="s">
@@ -3776,7 +3783,7 @@
       <c r="M6">
         <v>1171</v>
       </c>
-      <c r="N6" t="s">
+      <c r="N6" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O6" t="s">
@@ -3889,7 +3896,7 @@
       <c r="M7">
         <v>712</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N7" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O7" t="s">
@@ -4002,7 +4009,7 @@
       <c r="M8">
         <v>712</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N8" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O8" t="s">
@@ -4115,7 +4122,7 @@
       <c r="M9">
         <v>1193</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O9" t="s">
@@ -4228,7 +4235,7 @@
       <c r="M10">
         <v>1171</v>
       </c>
-      <c r="N10" t="s">
+      <c r="N10" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O10" t="s">
@@ -4341,7 +4348,7 @@
       <c r="M11">
         <v>712</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N11" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O11" t="s">
@@ -4454,7 +4461,7 @@
       <c r="M12">
         <v>1309</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N12" s="4" t="s">
         <v>242</v>
       </c>
       <c r="O12" t="s">
@@ -4567,7 +4574,7 @@
       <c r="M13">
         <v>1171</v>
       </c>
-      <c r="N13" t="s">
+      <c r="N13" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O13" t="s">
@@ -4680,7 +4687,7 @@
       <c r="M14">
         <v>712</v>
       </c>
-      <c r="N14" t="s">
+      <c r="N14" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O14" t="s">
@@ -4793,7 +4800,7 @@
       <c r="M15">
         <v>1193</v>
       </c>
-      <c r="N15" t="s">
+      <c r="N15" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O15" t="s">
@@ -4906,7 +4913,7 @@
       <c r="M16">
         <v>712</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N16" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O16" t="s">
@@ -5019,7 +5026,7 @@
       <c r="M17">
         <v>1171</v>
       </c>
-      <c r="N17" t="s">
+      <c r="N17" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O17" t="s">
@@ -5132,7 +5139,7 @@
       <c r="M18">
         <v>712</v>
       </c>
-      <c r="N18" t="s">
+      <c r="N18" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O18" t="s">
@@ -5245,7 +5252,7 @@
       <c r="M19">
         <v>1171</v>
       </c>
-      <c r="N19" t="s">
+      <c r="N19" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O19" t="s">
@@ -5358,7 +5365,7 @@
       <c r="M20">
         <v>712</v>
       </c>
-      <c r="N20" t="s">
+      <c r="N20" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O20" t="s">
@@ -5471,7 +5478,7 @@
       <c r="M21">
         <v>1193</v>
       </c>
-      <c r="N21" t="s">
+      <c r="N21" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O21" t="s">
@@ -5584,7 +5591,7 @@
       <c r="M22">
         <v>1171</v>
       </c>
-      <c r="N22" t="s">
+      <c r="N22" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O22" t="s">
@@ -5697,7 +5704,7 @@
       <c r="M23">
         <v>1309</v>
       </c>
-      <c r="N23" t="s">
+      <c r="N23" s="4" t="s">
         <v>242</v>
       </c>
       <c r="O23" t="s">
@@ -5810,7 +5817,7 @@
       <c r="M24">
         <v>712</v>
       </c>
-      <c r="N24" t="s">
+      <c r="N24" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O24" t="s">
@@ -5923,7 +5930,7 @@
       <c r="M25">
         <v>1171</v>
       </c>
-      <c r="N25" t="s">
+      <c r="N25" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O25" t="s">
@@ -6036,7 +6043,7 @@
       <c r="M26">
         <v>1193</v>
       </c>
-      <c r="N26" t="s">
+      <c r="N26" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O26" t="s">
@@ -6149,7 +6156,7 @@
       <c r="M27">
         <v>1171</v>
       </c>
-      <c r="N27" t="s">
+      <c r="N27" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O27" t="s">
@@ -6262,7 +6269,7 @@
       <c r="M28">
         <v>712</v>
       </c>
-      <c r="N28" t="s">
+      <c r="N28" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O28" t="s">
@@ -6375,7 +6382,7 @@
       <c r="M29">
         <v>1171</v>
       </c>
-      <c r="N29" t="s">
+      <c r="N29" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O29" t="s">
@@ -6488,7 +6495,7 @@
       <c r="M30">
         <v>1171</v>
       </c>
-      <c r="N30" t="s">
+      <c r="N30" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O30" t="s">
@@ -6601,7 +6608,7 @@
       <c r="M31">
         <v>1193</v>
       </c>
-      <c r="N31" t="s">
+      <c r="N31" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O31" t="s">
@@ -6714,7 +6721,7 @@
       <c r="M32">
         <v>1171</v>
       </c>
-      <c r="N32" t="s">
+      <c r="N32" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O32" t="s">
@@ -6827,7 +6834,7 @@
       <c r="M33">
         <v>1171</v>
       </c>
-      <c r="N33" t="s">
+      <c r="N33" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O33" t="s">
@@ -6940,7 +6947,7 @@
       <c r="M34">
         <v>1195</v>
       </c>
-      <c r="N34" t="s">
+      <c r="N34" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O34" t="s">
@@ -7053,7 +7060,7 @@
       <c r="M35">
         <v>1309</v>
       </c>
-      <c r="N35" t="s">
+      <c r="N35" s="4" t="s">
         <v>242</v>
       </c>
       <c r="O35" t="s">
@@ -7166,7 +7173,7 @@
       <c r="M36">
         <v>1171</v>
       </c>
-      <c r="N36" t="s">
+      <c r="N36" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O36" t="s">
@@ -7279,7 +7286,7 @@
       <c r="M37">
         <v>1171</v>
       </c>
-      <c r="N37" t="s">
+      <c r="N37" s="4" t="s">
         <v>222</v>
       </c>
       <c r="O37" t="s">
@@ -7392,7 +7399,7 @@
       <c r="M38">
         <v>712</v>
       </c>
-      <c r="N38" t="s">
+      <c r="N38" s="4" t="s">
         <v>208</v>
       </c>
       <c r="O38" t="s">
@@ -7505,7 +7512,7 @@
       <c r="M39">
         <v>1193</v>
       </c>
-      <c r="N39" t="s">
+      <c r="N39" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O39" t="s">
@@ -7618,7 +7625,7 @@
       <c r="M40">
         <v>1309</v>
       </c>
-      <c r="N40" t="s">
+      <c r="N40" s="4" t="s">
         <v>242</v>
       </c>
       <c r="O40" t="s">
@@ -7731,7 +7738,7 @@
       <c r="M41">
         <v>1193</v>
       </c>
-      <c r="N41" t="s">
+      <c r="N41" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O41" t="s">
@@ -7844,7 +7851,7 @@
       <c r="M42">
         <v>1309</v>
       </c>
-      <c r="N42" t="s">
+      <c r="N42" s="4" t="s">
         <v>242</v>
       </c>
       <c r="O42" t="s">
@@ -7957,7 +7964,7 @@
       <c r="M43">
         <v>1193</v>
       </c>
-      <c r="N43" t="s">
+      <c r="N43" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O43" t="s">
@@ -8070,7 +8077,7 @@
       <c r="M44">
         <v>1193</v>
       </c>
-      <c r="N44" t="s">
+      <c r="N44" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O44" t="s">
@@ -8183,7 +8190,7 @@
       <c r="M45">
         <v>1193</v>
       </c>
-      <c r="N45" t="s">
+      <c r="N45" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O45" t="s">
@@ -8296,7 +8303,7 @@
       <c r="M46">
         <v>1193</v>
       </c>
-      <c r="N46" t="s">
+      <c r="N46" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O46" t="s">
@@ -8409,7 +8416,7 @@
       <c r="M47">
         <v>1193</v>
       </c>
-      <c r="N47" t="s">
+      <c r="N47" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O47" t="s">
@@ -8522,7 +8529,7 @@
       <c r="M48">
         <v>1193</v>
       </c>
-      <c r="N48" t="s">
+      <c r="N48" s="4" t="s">
         <v>235</v>
       </c>
       <c r="O48" t="s">

</xml_diff>